<commit_message>
Informe actualizado - Gráfico desfasaje pendiente de revisión
</commit_message>
<xml_diff>
--- a/Matlab - Simulink/Tablas/Tabla_Polos_Temperatura.xlsx
+++ b/Matlab - Simulink/Tablas/Tabla_Polos_Temperatura.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>Rs_Ohm</t>
   </si>
@@ -24,10 +24,175 @@
     <t>P2</t>
   </si>
   <si>
+    <t>-95.34424+145.7293i</t>
+  </si>
+  <si>
+    <t>-98.77355+143.4537i</t>
+  </si>
+  <si>
+    <t>-102.2029+141.058i</t>
+  </si>
+  <si>
+    <t>-105.6322+138.536i</t>
+  </si>
+  <si>
+    <t>-109.0615+135.8808i</t>
+  </si>
+  <si>
+    <t>-112.4908+133.0842i</t>
+  </si>
+  <si>
+    <t>-115.9201+130.1374i</t>
+  </si>
+  <si>
+    <t>-119.3494+127.0296i</t>
+  </si>
+  <si>
     <t>P3</t>
   </si>
   <si>
+    <t>-95.34424-145.7293i</t>
+  </si>
+  <si>
+    <t>-98.77355-143.4537i</t>
+  </si>
+  <si>
+    <t>-102.2029-141.058i</t>
+  </si>
+  <si>
+    <t>-105.6322-138.536i</t>
+  </si>
+  <si>
+    <t>-109.0615-135.8808i</t>
+  </si>
+  <si>
+    <t>-112.4908-133.0842i</t>
+  </si>
+  <si>
+    <t>-115.9201-130.1374i</t>
+  </si>
+  <si>
+    <t>-119.3494-127.0296i</t>
+  </si>
+  <si>
     <t>Ceros</t>
+  </si>
+  <si>
+    <t>-189.5793</t>
+  </si>
+  <si>
+    <t>-196.4379</t>
+  </si>
+  <si>
+    <t>-203.2966</t>
+  </si>
+  <si>
+    <t>-210.1552</t>
+  </si>
+  <si>
+    <t>-217.0138</t>
+  </si>
+  <si>
+    <t>-223.8724</t>
+  </si>
+  <si>
+    <t>-230.731</t>
+  </si>
+  <si>
+    <t>-237.5897</t>
+  </si>
+  <si>
+    <t>wn_rad_s</t>
+  </si>
+  <si>
+    <t>zeta</t>
+  </si>
+  <si>
+    <t>Rs_Ohm</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>-95.34424+145.7293i</t>
+  </si>
+  <si>
+    <t>-98.77355+143.4537i</t>
+  </si>
+  <si>
+    <t>-102.2029+141.058i</t>
+  </si>
+  <si>
+    <t>-105.6322+138.536i</t>
+  </si>
+  <si>
+    <t>-109.0615+135.8808i</t>
+  </si>
+  <si>
+    <t>-112.4908+133.0842i</t>
+  </si>
+  <si>
+    <t>-115.9201+130.1374i</t>
+  </si>
+  <si>
+    <t>-119.3494+127.0296i</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>-95.34424-145.7293i</t>
+  </si>
+  <si>
+    <t>-98.77355-143.4537i</t>
+  </si>
+  <si>
+    <t>-102.2029-141.058i</t>
+  </si>
+  <si>
+    <t>-105.6322-138.536i</t>
+  </si>
+  <si>
+    <t>-109.0615-135.8808i</t>
+  </si>
+  <si>
+    <t>-112.4908-133.0842i</t>
+  </si>
+  <si>
+    <t>-115.9201-130.1374i</t>
+  </si>
+  <si>
+    <t>-119.3494-127.0296i</t>
+  </si>
+  <si>
+    <t>Ceros</t>
+  </si>
+  <si>
+    <t>-189.5793</t>
+  </si>
+  <si>
+    <t>-196.4379</t>
+  </si>
+  <si>
+    <t>-203.2966</t>
+  </si>
+  <si>
+    <t>-210.1552</t>
+  </si>
+  <si>
+    <t>-217.0138</t>
+  </si>
+  <si>
+    <t>-223.8724</t>
+  </si>
+  <si>
+    <t>-230.731</t>
+  </si>
+  <si>
+    <t>-237.5897</t>
   </si>
   <si>
     <t>wn_rad_s</t>
@@ -279,25 +444,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>38</v>
+        <v>93</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>58</v>
+        <v>113</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>67</v>
+        <v>122</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>68</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
@@ -308,13 +473,13 @@
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>41</v>
+        <v>96</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>50</v>
+        <v>105</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>59</v>
+        <v>114</v>
       </c>
       <c r="F2" s="0">
         <v>174.14808792866981</v>
@@ -331,13 +496,13 @@
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>42</v>
+        <v>97</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>51</v>
+        <v>106</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>60</v>
+        <v>115</v>
       </c>
       <c r="F3" s="0">
         <v>174.16992807182058</v>
@@ -354,13 +519,13 @@
         <v>0</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>43</v>
+        <v>98</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="F4" s="0">
         <v>174.19176547665683</v>
@@ -377,13 +542,13 @@
         <v>0</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>44</v>
+        <v>99</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>62</v>
+        <v>117</v>
       </c>
       <c r="F5" s="0">
         <v>174.21360014420821</v>
@@ -400,13 +565,13 @@
         <v>0</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="F6" s="0">
         <v>174.23543207550384</v>
@@ -423,13 +588,13 @@
         <v>0</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>46</v>
+        <v>101</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="F7" s="0">
         <v>174.25726127157219</v>
@@ -446,13 +611,13 @@
         <v>0</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>47</v>
+        <v>102</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="F8" s="0">
         <v>174.279087733441</v>
@@ -469,13 +634,13 @@
         <v>0</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>48</v>
+        <v>103</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>66</v>
+        <v>121</v>
       </c>
       <c r="F9" s="0">
         <v>174.30091146213746</v>

</xml_diff>